<commit_message>
implementacion del TDD, edicion de nombre de archivo final, seleccion de inputs para enviar a la ia, mejora de UI
</commit_message>
<xml_diff>
--- a/templates/TDD.xlsx
+++ b/templates/TDD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mvidaurre\Desktop\RPA\documentAssistant\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD9E5C0-DDB7-419E-AD3F-66F3DCF6080D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702FD6D3-F26D-4EE6-A482-1677C4F28FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -671,7 +671,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -786,9 +786,6 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -815,50 +812,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -1158,21 +1112,21 @@
       </c>
     </row>
     <row r="6" spans="2:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
-      <c r="M6" s="47"/>
-      <c r="N6" s="47"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="46"/>
+      <c r="I6" s="46"/>
+      <c r="J6" s="46"/>
+      <c r="K6" s="46"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="46"/>
+      <c r="N6" s="46"/>
     </row>
     <row r="7" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="28" t="s">
@@ -1207,13 +1161,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
     </row>
     <row r="3" spans="1:5" s="6" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -1222,47 +1176,47 @@
       <c r="C3" s="23"/>
     </row>
     <row r="4" spans="1:5" s="5" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="52"/>
+      <c r="B4" s="51"/>
       <c r="C4" s="20" t="str">
         <f ca="1">MID(CELL("filename"),FIND("[",CELL("filename"))+1,FIND("]",CELL("filename"))-FIND("[",CELL("filename"))-1)</f>
         <v>TDD.xlsx</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="5" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="52"/>
+      <c r="B5" s="51"/>
       <c r="C5" s="20" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="5" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="51" t="s">
+      <c r="A6" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="52"/>
+      <c r="B6" s="51"/>
       <c r="C6" s="20" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="5" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="51" t="s">
+      <c r="A7" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="52"/>
+      <c r="B7" s="51"/>
       <c r="C7" s="20" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="5" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="52"/>
+      <c r="B8" s="51"/>
       <c r="C8" s="22" t="s">
         <v>17</v>
       </c>
@@ -1298,16 +1252,16 @@
       <c r="C12" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="53" t="s">
+      <c r="D12" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="54"/>
+      <c r="E12" s="53"/>
     </row>
     <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A13"/>
       <c r="C13" s="21"/>
-      <c r="D13" s="50"/>
-      <c r="E13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1415,7 +1369,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
         <v>44</v>
       </c>
@@ -1423,7 +1377,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>46</v>
       </c>
@@ -1432,14 +1386,14 @@
       </c>
     </row>
     <row r="6" spans="1:6" s="17" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
     </row>
     <row r="7" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="30"/>
@@ -1503,8 +1457,9 @@
     <col min="1" max="1" width="31.28515625" style="2" customWidth="1"/>
     <col min="2" max="2" width="40.140625" style="2" customWidth="1"/>
     <col min="3" max="3" width="28.7109375" style="2" customWidth="1"/>
-    <col min="4" max="5" width="34.7109375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="19.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="33.140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="35.42578125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" style="2" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
@@ -1524,7 +1479,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
         <v>44</v>
       </c>
@@ -1532,7 +1487,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="43" t="s">
         <v>46</v>
       </c>
@@ -1545,14 +1500,14 @@
       <c r="B5" s="16"/>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
     </row>
     <row r="7" spans="1:6" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="30"/>
@@ -1572,12 +1527,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="38"/>
       <c r="B8" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="40" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="36" t="s">
@@ -1586,7 +1541,7 @@
       <c r="E8" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="35" t="s">
+      <c r="F8" s="36" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>